<commit_message>
add Minitab instructions and update Class 5 schedule with activities
</commit_message>
<xml_diff>
--- a/math121-schedule.xlsx
+++ b/math121-schedule.xlsx
@@ -742,6 +742,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -779,21 +794,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1155,7 +1155,7 @@
       <c r="C2" s="15">
         <v>46265</v>
       </c>
-      <c r="D2" s="51" t="s">
+      <c r="D2" s="38" t="s">
         <v>46</v>
       </c>
       <c r="E2" s="6" t="s">
@@ -1173,7 +1173,7 @@
         <f>C2+3</f>
         <v>46268</v>
       </c>
-      <c r="D3" s="51"/>
+      <c r="D3" s="38"/>
       <c r="E3" s="6" t="s">
         <v>5</v>
       </c>
@@ -1242,7 +1242,7 @@
         <f t="shared" ref="C6:C35" si="2">C4+7</f>
         <v>46279</v>
       </c>
-      <c r="D6" s="51" t="s">
+      <c r="D6" s="38" t="s">
         <v>49</v>
       </c>
       <c r="E6" s="6" t="s">
@@ -1265,7 +1265,7 @@
         <f t="shared" si="2"/>
         <v>46282</v>
       </c>
-      <c r="D7" s="51"/>
+      <c r="D7" s="38"/>
       <c r="E7" s="6" t="s">
         <v>9</v>
       </c>
@@ -1287,7 +1287,7 @@
         <f t="shared" si="2"/>
         <v>46286</v>
       </c>
-      <c r="D8" s="51" t="s">
+      <c r="D8" s="38" t="s">
         <v>50</v>
       </c>
       <c r="E8" s="6" t="s">
@@ -1310,7 +1310,7 @@
         <f t="shared" si="2"/>
         <v>46289</v>
       </c>
-      <c r="D9" s="51"/>
+      <c r="D9" s="38"/>
       <c r="E9" s="6" t="s">
         <v>11</v>
       </c>
@@ -1349,12 +1349,12 @@
       <c r="C11" s="15">
         <v>46294</v>
       </c>
-      <c r="D11" s="52" t="s">
+      <c r="D11" s="39" t="s">
         <v>79</v>
       </c>
-      <c r="E11" s="52"/>
-      <c r="F11" s="52"/>
-      <c r="G11" s="52"/>
+      <c r="E11" s="39"/>
+      <c r="F11" s="39"/>
+      <c r="G11" s="39"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="9"/>
@@ -1388,7 +1388,7 @@
         <f>C10+7</f>
         <v>46300</v>
       </c>
-      <c r="D13" s="51" t="s">
+      <c r="D13" s="38" t="s">
         <v>51</v>
       </c>
       <c r="E13" s="6" t="s">
@@ -1409,7 +1409,7 @@
         <f t="shared" si="2"/>
         <v>46303</v>
       </c>
-      <c r="D14" s="51"/>
+      <c r="D14" s="38"/>
       <c r="E14" s="6" t="s">
         <v>15</v>
       </c>
@@ -1429,7 +1429,7 @@
         <f t="shared" si="2"/>
         <v>46307</v>
       </c>
-      <c r="D15" s="51" t="s">
+      <c r="D15" s="38" t="s">
         <v>52</v>
       </c>
       <c r="E15" s="6" t="s">
@@ -1452,7 +1452,7 @@
         <f t="shared" si="2"/>
         <v>46310</v>
       </c>
-      <c r="D16" s="51"/>
+      <c r="D16" s="38"/>
       <c r="E16" s="6" t="s">
         <v>17</v>
       </c>
@@ -1488,7 +1488,7 @@
         <f t="shared" si="2"/>
         <v>46317</v>
       </c>
-      <c r="D18" s="51" t="s">
+      <c r="D18" s="38" t="s">
         <v>53</v>
       </c>
       <c r="E18" s="6" t="s">
@@ -1511,7 +1511,7 @@
         <f t="shared" si="2"/>
         <v>46321</v>
       </c>
-      <c r="D19" s="51"/>
+      <c r="D19" s="38"/>
       <c r="E19" s="6" t="s">
         <v>19</v>
       </c>
@@ -1526,23 +1526,23 @@
       <c r="C20" s="15">
         <v>46322</v>
       </c>
-      <c r="D20" s="53" t="s">
+      <c r="D20" s="40" t="s">
         <v>80</v>
       </c>
-      <c r="E20" s="54"/>
-      <c r="F20" s="54"/>
-      <c r="G20" s="55"/>
+      <c r="E20" s="41"/>
+      <c r="F20" s="41"/>
+      <c r="G20" s="42"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="9">
         <f>A18+1</f>
         <v>9</v>
       </c>
-      <c r="B21" s="38" t="str">
+      <c r="B21" s="43" t="str">
         <f>B18</f>
         <v>Thu</v>
       </c>
-      <c r="C21" s="40">
+      <c r="C21" s="45">
         <f>C18+7</f>
         <v>46324</v>
       </c>
@@ -1559,14 +1559,14 @@
     </row>
     <row r="22" spans="1:7" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="9"/>
-      <c r="B22" s="39"/>
-      <c r="C22" s="41"/>
-      <c r="D22" s="42" t="s">
+      <c r="B22" s="44"/>
+      <c r="C22" s="46"/>
+      <c r="D22" s="47" t="s">
         <v>81</v>
       </c>
-      <c r="E22" s="43"/>
-      <c r="F22" s="43"/>
-      <c r="G22" s="44"/>
+      <c r="E22" s="48"/>
+      <c r="F22" s="48"/>
+      <c r="G22" s="49"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="9"/>
@@ -1600,7 +1600,7 @@
         <f>C21+7</f>
         <v>46331</v>
       </c>
-      <c r="D24" s="51" t="s">
+      <c r="D24" s="38" t="s">
         <v>54</v>
       </c>
       <c r="E24" s="6" t="s">
@@ -1621,7 +1621,7 @@
         <f t="shared" si="2"/>
         <v>46335</v>
       </c>
-      <c r="D25" s="51"/>
+      <c r="D25" s="38"/>
       <c r="E25" s="6" t="s">
         <v>23</v>
       </c>
@@ -1629,7 +1629,7 @@
       <c r="G25" s="13"/>
     </row>
     <row r="26" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="45">
+      <c r="A26" s="50">
         <f>A24+1</f>
         <v>11</v>
       </c>
@@ -1639,15 +1639,15 @@
       <c r="C26" s="15">
         <v>46337</v>
       </c>
-      <c r="D26" s="48" t="s">
+      <c r="D26" s="53" t="s">
         <v>83</v>
       </c>
-      <c r="E26" s="49"/>
-      <c r="F26" s="49"/>
-      <c r="G26" s="50"/>
+      <c r="E26" s="54"/>
+      <c r="F26" s="54"/>
+      <c r="G26" s="55"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="46"/>
+      <c r="A27" s="51"/>
       <c r="B27" s="17" t="str">
         <f>B24</f>
         <v>Thu</v>
@@ -1656,7 +1656,7 @@
         <f>C24+7</f>
         <v>46338</v>
       </c>
-      <c r="D27" s="51" t="s">
+      <c r="D27" s="38" t="s">
         <v>55</v>
       </c>
       <c r="E27" s="6" t="s">
@@ -1670,7 +1670,7 @@
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="47"/>
+      <c r="A28" s="52"/>
       <c r="B28" s="17" t="str">
         <f>B25</f>
         <v>Mon</v>
@@ -1679,7 +1679,7 @@
         <f>C25+7</f>
         <v>46342</v>
       </c>
-      <c r="D28" s="51"/>
+      <c r="D28" s="38"/>
       <c r="E28" s="6" t="s">
         <v>25</v>
       </c>
@@ -1699,7 +1699,7 @@
         <f t="shared" si="2"/>
         <v>46345</v>
       </c>
-      <c r="D29" s="51" t="s">
+      <c r="D29" s="38" t="s">
         <v>76</v>
       </c>
       <c r="E29" s="6" t="s">
@@ -1720,7 +1720,7 @@
         <f t="shared" si="2"/>
         <v>46349</v>
       </c>
-      <c r="D30" s="51"/>
+      <c r="D30" s="38"/>
       <c r="E30" s="6" t="s">
         <v>27</v>
       </c>
@@ -1801,7 +1801,7 @@
         <f t="shared" si="2"/>
         <v>46363</v>
       </c>
-      <c r="D34" s="51" t="s">
+      <c r="D34" s="38" t="s">
         <v>45</v>
       </c>
       <c r="E34" s="6" t="s">
@@ -1822,7 +1822,7 @@
         <f t="shared" si="2"/>
         <v>46366</v>
       </c>
-      <c r="D35" s="51"/>
+      <c r="D35" s="38"/>
       <c r="E35" s="6" t="s">
         <v>31</v>
       </c>
@@ -1856,6 +1856,11 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="C21:C22"/>
+    <mergeCell ref="D22:G22"/>
+    <mergeCell ref="A26:A28"/>
+    <mergeCell ref="D26:G26"/>
     <mergeCell ref="D29:D30"/>
     <mergeCell ref="D34:D35"/>
     <mergeCell ref="D8:D9"/>
@@ -1868,11 +1873,6 @@
     <mergeCell ref="D27:D28"/>
     <mergeCell ref="D11:G11"/>
     <mergeCell ref="D20:G20"/>
-    <mergeCell ref="B21:B22"/>
-    <mergeCell ref="C21:C22"/>
-    <mergeCell ref="D22:G22"/>
-    <mergeCell ref="A26:A28"/>
-    <mergeCell ref="D26:G26"/>
   </mergeCells>
   <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>